<commit_message>
feat: compile xlsx into a module
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,36 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Informatica\Desktop\Angel\src\calculadora-pruebas\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tecnesp\DocumentosTecnesp\angelf\Source\calculadora-pruebas\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9ECBCBE-2971-4D2B-8534-08336507285A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD82B1DE-C028-4ED1-B6A4-95E433A1D713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="3" r:id="rId1"/>
     <sheet name="Examenes" sheetId="1" r:id="rId2"/>
     <sheet name="Perfiles" sheetId="2" r:id="rId3"/>
+    <sheet name="ExcelOptions" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="126">
   <si>
     <t>last_edited</t>
   </si>
@@ -50,16 +48,373 @@
     <t>aliases</t>
   </si>
   <si>
-    <t>special_price</t>
-  </si>
-  <si>
-    <t>exam_ids</t>
+    <t>category</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>examIds</t>
+  </si>
+  <si>
+    <t>specialPrice</t>
+  </si>
+  <si>
+    <t>% DE SATURACION</t>
+  </si>
+  <si>
+    <t>ACIDO URICO</t>
+  </si>
+  <si>
+    <t>ACS. PARA TUBERCULOSIS</t>
+  </si>
+  <si>
+    <t>AG. HELICOBACTER PILORY (HECES)</t>
+  </si>
+  <si>
+    <t>AGLUTININAS ANTI RH</t>
+  </si>
+  <si>
+    <t>AGLUTININAS FEBRILES</t>
+  </si>
+  <si>
+    <t>AMILASA</t>
+  </si>
+  <si>
+    <t>ANTI D.N.A</t>
+  </si>
+  <si>
+    <t>ANTICUERPOS ANTINUCLEARES</t>
+  </si>
+  <si>
+    <t>ANTICUERPOS TOXOPLASMICOS (HAI)</t>
+  </si>
+  <si>
+    <t>ANTIESTREPTOLISINA O</t>
+  </si>
+  <si>
+    <t>B.H.C.G. CUANTITATIVA</t>
+  </si>
+  <si>
+    <t>BILIRRUBINA</t>
+  </si>
+  <si>
+    <t>CALCIO</t>
+  </si>
+  <si>
+    <t>CARDIOLIPINA IgG-IgM</t>
+  </si>
+  <si>
+    <t>CCP. CITRULINADO</t>
+  </si>
+  <si>
+    <t>CELULAS L.E.</t>
+  </si>
+  <si>
+    <t>CHAGAS</t>
+  </si>
+  <si>
+    <t>CITOMEGALOVIRUS IgG-IgM</t>
+  </si>
+  <si>
+    <t>CLORO</t>
+  </si>
+  <si>
+    <t>COLESTEROL</t>
+  </si>
+  <si>
+    <t>COOMBS DIRECTO</t>
+  </si>
+  <si>
+    <t>COOMBS INDIRECTO</t>
+  </si>
+  <si>
+    <t>CORTISOL</t>
+  </si>
+  <si>
+    <t>Hormona del estrés</t>
+  </si>
+  <si>
+    <t>CREATININA</t>
+  </si>
+  <si>
+    <t>CULTIVOS (UROCULTIVO, HEMOCULTIVO, ETC)</t>
+  </si>
+  <si>
+    <t>DENGUE (IgG-IgM)</t>
+  </si>
+  <si>
+    <t>DEP. DE CREATININA EN 24 H.</t>
+  </si>
+  <si>
+    <t>DHEA-S</t>
+  </si>
+  <si>
+    <t>EPSTEIN BARR IgG-IgM</t>
+  </si>
+  <si>
+    <t>ESTRADIOL</t>
+  </si>
+  <si>
+    <t>EX. HECES</t>
+  </si>
+  <si>
+    <t>F.S.H.</t>
+  </si>
+  <si>
+    <t>FACTOR REUMATOIDEO LATEX</t>
+  </si>
+  <si>
+    <t>FENOMENO LE</t>
+  </si>
+  <si>
+    <t>FIBRINOGENO</t>
+  </si>
+  <si>
+    <t>FOSFATASA ALCALINA</t>
+  </si>
+  <si>
+    <t>FOSFOLIPIDOS IgG-IgM</t>
+  </si>
+  <si>
+    <t>FOSFORO</t>
+  </si>
+  <si>
+    <t>FROTIS DE SANGRE PERIFERICA</t>
+  </si>
+  <si>
+    <t>G.G.T</t>
+  </si>
+  <si>
+    <t>GLICEMIA</t>
+  </si>
+  <si>
+    <t>GLICEMIA POST PANDRIAL</t>
+  </si>
+  <si>
+    <t>GRUPO SANGUINEO</t>
+  </si>
+  <si>
+    <t>HEMOGLOBINA GLICADA (HbA1c)</t>
+  </si>
+  <si>
+    <t>HELICOBACTER PYLORI CUALITATIVO</t>
+  </si>
+  <si>
+    <t>HELICOBACTER PYLORI IgG-IgM</t>
+  </si>
+  <si>
+    <t>HEMATOLOGIA COMPLETA</t>
+  </si>
+  <si>
+    <t>Hemograma</t>
+  </si>
+  <si>
+    <t>HEMOCULTIVO</t>
+  </si>
+  <si>
+    <t>CULT LIQ</t>
+  </si>
+  <si>
+    <t>COPROCULTIVO</t>
+  </si>
+  <si>
+    <t>HEPATITIS A IgG</t>
+  </si>
+  <si>
+    <t>HEPATITIS A IgM</t>
+  </si>
+  <si>
+    <t>HIERRO</t>
+  </si>
+  <si>
+    <t>HIV 1+2 ELISA (4TA. GEN.)</t>
+  </si>
+  <si>
+    <t>INMUNOGLOBULINA A</t>
+  </si>
+  <si>
+    <t>INMUNOGLOBULINA E (IGE)</t>
+  </si>
+  <si>
+    <t>INMUNOGLOBULINA G</t>
+  </si>
+  <si>
+    <t>INMUNOGLOBULINA M</t>
+  </si>
+  <si>
+    <t>L.H</t>
+  </si>
+  <si>
+    <t>LDH</t>
+  </si>
+  <si>
+    <t>LEUCOCITOS</t>
+  </si>
+  <si>
+    <t>DIFERENCIAL</t>
+  </si>
+  <si>
+    <t>LIPASA</t>
+  </si>
+  <si>
+    <t>MAGNESIO</t>
+  </si>
+  <si>
+    <t>MICROALBUMINURIA</t>
+  </si>
+  <si>
+    <t>ORINA</t>
+  </si>
+  <si>
+    <t>PCR CUANTITATIVA</t>
+  </si>
+  <si>
+    <t>PERFIL LIPIDICO</t>
+  </si>
+  <si>
+    <t>PERFIL TIROIDEO</t>
+  </si>
+  <si>
+    <t>PERFIL TORCH (CMV, RUBEOLA, HERPES, TOXO)</t>
+  </si>
+  <si>
+    <t>PERFIL PROSTÁTICO</t>
+  </si>
+  <si>
+    <t>PH y AZUCARES RED.</t>
+  </si>
+  <si>
+    <t>POTASIO</t>
+  </si>
+  <si>
+    <t>PROGESTERONA</t>
+  </si>
+  <si>
+    <t>PROLACTINA</t>
+  </si>
+  <si>
+    <t>PROTEINURIA</t>
+  </si>
+  <si>
+    <t>PROTEOGRAMA</t>
+  </si>
+  <si>
+    <t>PRUEBA DE EMBARAZO CUALITATIVA</t>
+  </si>
+  <si>
+    <t>PRUEBA de IGRA PARA TUBERCULOSIS</t>
+  </si>
+  <si>
+    <t>REL. ACIDO URICO/CREATININA</t>
+  </si>
+  <si>
+    <t>REL. CALCIO/CREATININA</t>
+  </si>
+  <si>
+    <t>RETICULOCITO</t>
+  </si>
+  <si>
+    <t>SANGRE OCULTA (HECES)</t>
+  </si>
+  <si>
+    <t>SODIO</t>
+  </si>
+  <si>
+    <t>SUDAM III (HECES)</t>
+  </si>
+  <si>
+    <t>TIEMPO DE SANGRIA</t>
+  </si>
+  <si>
+    <t>TIEMPO DE COAGULACION</t>
+  </si>
+  <si>
+    <t>T.G.O</t>
+  </si>
+  <si>
+    <t>T.G.P</t>
+  </si>
+  <si>
+    <t>T.P.T</t>
+  </si>
+  <si>
+    <t>T.P</t>
+  </si>
+  <si>
+    <t>T.S.H</t>
+  </si>
+  <si>
+    <t>T3 LIBRE</t>
+  </si>
+  <si>
+    <t>T3 TOTAL</t>
+  </si>
+  <si>
+    <t>T4 LIBRE</t>
+  </si>
+  <si>
+    <t>T4 TOTAL</t>
+  </si>
+  <si>
+    <t>TESTOSTERONA LIBRE</t>
+  </si>
+  <si>
+    <t>TESTOSTERONA TOTAL</t>
+  </si>
+  <si>
+    <t>TOXO (IgG-IgM)</t>
+  </si>
+  <si>
+    <t>TRANSFERRINA</t>
+  </si>
+  <si>
+    <t>TRIGLICERIDOS</t>
+  </si>
+  <si>
+    <t>UREA</t>
+  </si>
+  <si>
+    <t>V.S.G</t>
+  </si>
+  <si>
+    <t>VDRL</t>
+  </si>
+  <si>
+    <t>S: Serología</t>
+  </si>
+  <si>
+    <t>Q: Química</t>
+  </si>
+  <si>
+    <t>B: Bacteriología</t>
+  </si>
+  <si>
+    <t>A: Pruebas de Alergia</t>
+  </si>
+  <si>
+    <t>H: Hormonas</t>
+  </si>
+  <si>
+    <t>U: Uroanálisis</t>
+  </si>
+  <si>
+    <t>C: Coproanálisis</t>
+  </si>
+  <si>
+    <t>MT: Marcadores Tumorales</t>
+  </si>
+  <si>
+    <t>O: Otros</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -105,10 +460,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,7 +757,7 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -412,15 +768,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -432,23 +789,1201 @@
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25">
+        <v>35</v>
+      </c>
+      <c r="D25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>46</v>
+      </c>
+      <c r="C37">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>49</v>
+      </c>
+      <c r="C40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>52</v>
+      </c>
+      <c r="C43">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>53</v>
+      </c>
+      <c r="C44">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>54</v>
+      </c>
+      <c r="C45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49">
+        <v>8</v>
+      </c>
+      <c r="D49" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>60</v>
+      </c>
+      <c r="C50">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>62</v>
+      </c>
+      <c r="C52">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>63</v>
+      </c>
+      <c r="C53">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>66</v>
+      </c>
+      <c r="C56">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>67</v>
+      </c>
+      <c r="C57">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>68</v>
+      </c>
+      <c r="C58">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>69</v>
+      </c>
+      <c r="C59">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>70</v>
+      </c>
+      <c r="C60">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>71</v>
+      </c>
+      <c r="C61">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>72</v>
+      </c>
+      <c r="C62">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>73</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>75</v>
+      </c>
+      <c r="C65">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>76</v>
+      </c>
+      <c r="C66">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>77</v>
+      </c>
+      <c r="C67">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>78</v>
+      </c>
+      <c r="C68">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>79</v>
+      </c>
+      <c r="C69">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>80</v>
+      </c>
+      <c r="C70">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>81</v>
+      </c>
+      <c r="C71">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>82</v>
+      </c>
+      <c r="C72">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>83</v>
+      </c>
+      <c r="C73">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>84</v>
+      </c>
+      <c r="C74">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>85</v>
+      </c>
+      <c r="C75">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>86</v>
+      </c>
+      <c r="C76">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>87</v>
+      </c>
+      <c r="C77">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>88</v>
+      </c>
+      <c r="C78">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>89</v>
+      </c>
+      <c r="C79">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>90</v>
+      </c>
+      <c r="C80">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>91</v>
+      </c>
+      <c r="C81">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>92</v>
+      </c>
+      <c r="C82">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>93</v>
+      </c>
+      <c r="C83">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>94</v>
+      </c>
+      <c r="C84">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>95</v>
+      </c>
+      <c r="C85">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>96</v>
+      </c>
+      <c r="C86">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>97</v>
+      </c>
+      <c r="C87">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>98</v>
+      </c>
+      <c r="C88">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>99</v>
+      </c>
+      <c r="C89">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>100</v>
+      </c>
+      <c r="C90">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>101</v>
+      </c>
+      <c r="C91">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>102</v>
+      </c>
+      <c r="C92">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>103</v>
+      </c>
+      <c r="C93">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>104</v>
+      </c>
+      <c r="C94">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>105</v>
+      </c>
+      <c r="C95">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>106</v>
+      </c>
+      <c r="C96">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>107</v>
+      </c>
+      <c r="C97">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>108</v>
+      </c>
+      <c r="C98">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>109</v>
+      </c>
+      <c r="C99">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>110</v>
+      </c>
+      <c r="C100">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>111</v>
+      </c>
+      <c r="C101">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>112</v>
+      </c>
+      <c r="C102">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>113</v>
+      </c>
+      <c r="C103">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>114</v>
+      </c>
+      <c r="C104">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>115</v>
+      </c>
+      <c r="C105">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>116</v>
+      </c>
+      <c r="C106">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B72CF788-15E2-4C61-8F02-096629DD74B4}">
+          <x14:formula1>
+            <xm:f>ExcelOptions!$A$2:$A$10</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B44F7564-083E-4685-B5C1-15DC42B07FF1}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -456,10 +1991,76 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F657691-98D5-4D60-833B-50CE0A68A732}">
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>